<commit_message>
feat(F-NAR-019): ATOM-COL.ECO.001-11 Le crayon de Sarah
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.ECO.001-11.xlsx
+++ b/stories/arbres/ATOM-COL.ECO.001-11.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>L'oiseau de papier de Sarah</t>
+          <t>Le crayon de Sarah</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cuisine, coin tapis, puis maison</t>
+          <t>école, coin tapis, vestiaire, puis maison</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Sarah, papa, maman, maîtresse</t>
+          <t>Sarah, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Un oiseau de papier pose sur la salière. Sarah veut lui dessiner une aile verte. Un chuchotement lui serre le ventre. Le soir, elle raconte, et l'oiseau gagne son aile.</t>
+          <t>Le vestiaire sent le pain du goûter. Sur le métal, un éclat de crochet tremble. Sarah veut dessiner, maintenant. Le crayon roule. À l'école, une voix trop près : malaise. Elle veut le dire tout de suite : les mots se cognent. Elle refuse de foncer, raconte au goûter. Merci vécu. Sur le métal, l'éclat tient.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un oiseau de papier pose sur la salière. Le papier fait un petit frou. Ça sent le pain grillé. Des miettes dorées sont sur la nappe. Un rayon touche l'aile pliée. La salière est un peu froide. Maman a plié l'oiseau ce matin. Il est léger, tu vois ? Oui, maman. Je veux lui dessiner une aile. Une aile verte. Tu pourras à l'école. Tu écoutes la maîtresse. Oui, papa. Les lacets sont bien faits. En ce moment, Sarah s'assoit. Le tapis a un carré d'or. Les cubes sont dans leur bac. On écoute. Ensuite, on range les crayons. Sarah aime écouter. Elle prend un crayon vert. Le bois est un peu râpeux. Elle dessine une aile, tout doux. L'aile a une petite plume. Le vert sent un peu le bois. C'est pour l'oiseau, maîtresse. Oui, Sarah. Tu as bien écouté. On range, maintenant. Sarah pose le crayon dans la boîte. L'aile verte reste sur la feuille. Plus tard, quelqu'un parle tout bas. Sarah entend parler d'un secret. Son ventre se serre. Elle pose la feuille près d'elle. Je raconterai à la maison. Le soir, papa coupe du pain. La croûte fait un petit bruit. Ça sent le four. Tu as faim, Sarah ? Sarah vient près de la planche. Elle a encore le ventre serré. L'oiseau de papier attend sur la salière.</t>
+          <t>Le vestiaire sent le pain du goûter. Les crochets portent des prénoms. Le prénom de Sarah est écrit. Un manteau rouge attend dans les bras. Les manches sont un peu froides. Maman lève le manteau vers le crochet. Le métal des crochets luit. Sur le métal, un éclat de crochet tremble. Il est petit, papa. C'est la lumière, sur le crochet. Papa accroche le manteau rouge. Le crochet tient le tissu. L'éclat de crochet brille, sous le manteau. Tes lacets sont faits, Sarah ? Oui, maman. Maman noue un lacet, puis l'autre. Les chaussures font un petit clac. Tu as senti le pain ? Oui, papa. Il sent le goûter. Sarah tient un crayon vert. Le bois est un peu râpeux. Je veux dessiner, maintenant ! Une maison, au coin tapis ? Oui, avec le crayon ! À tout à l'heure, Sarah. À tout à l'heure, papa. En ce moment, Sarah s'assoit. Le coin tapis est tiède. Un rayon fait un carré d'or. Les cubes attendent dans leur bac. La maîtresse parle près des chaises. Bonjour les enfants. Bonjour, maîtresse. Sarah veut le crayon, tout de suite. Elle ouvre la boîte trop vite. Le crayon roule sous un cube. Oh. Le sourire de Sarah disparaît. Elle reste près du groupe. Elle reprend le crayon, sans presser. Le bois est râpeux, un peu chaud. Je dessine la maison. Le vert sent le bois. La maison tient sur la feuille. Plus tard, une voix parle trop près. Sarah sent un malaise. Son ventre se serre, tout petit. Elle serre le crayon, puis le pose. Je le dirai à la maison. Le soir, le vestiaire est vide. Le manteau rouge revient. Papa coupe du pain. Ça sent le four. Te voilà. Tu as faim, Sarah ? Sarah veut le dire, tout de suite. Papa, à l'école ! Papa parle à maman, près du pain. Les mots de Sarah se cognent aux leurs. Personne ne tourne la tête. Tu disais quelque chose, Sarah ? Mon ventre s'est serré. Le sourire part, d'un coup. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne sort pas, maman. Ses épaules tombent un peu. Papa s'accroupit à sa hauteur. Tu veux du pain ? Sarah ouvre la bouche.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sylvain est à l'école. C'est le coin tapis. La maîtresse parle. Sylvain aime &lt;emphasis level="moderate"&gt;écouter&lt;/emphasis&gt;. Il écoute bien. La maîtresse dit : on range. Sylvain range un crayon. Plus tard, un camarade chuchote. Il dit : c'est un secret. Ne le dis pas à la maison. Sylvain sent un malaise. Son ventre est serré. Le soir, papa coupe du pain. Sylvain vient raconter à la maison. Il dit : papa, j'ai un malaise. Maman l'écoute aussi. Papa dit : tu as bien fait. On aime écouter la maîtresse. Si tu as un malaise, tu viens raconter.&lt;/prosody&gt;&lt;break time="400ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le vestiaire sent le pain du goûter. Les crochets portent des prénoms. Le prénom de Sarah est écrit. Un manteau rouge attend dans les bras. Les manches sont un peu froides. Maman lève le manteau vers le crochet. Le métal des crochets luit. Sur le métal, un &lt;emphasis level="moderate"&gt;éclat de crochet&lt;/emphasis&gt; tremble. Il est petit, papa. C'est la lumière, sur le crochet. Papa accroche le manteau rouge. Le crochet tient le tissu. L'éclat de crochet brille, sous le manteau. Tes lacets sont faits, Sarah ? Oui, maman. Maman noue un lacet, puis l'autre. Les chaussures font un petit clac. Tu as senti le pain ? Oui, papa. Il sent le goûter. Sarah tient un crayon vert. Le bois est un peu râpeux. Je veux dessiner, maintenant ! Une maison, au coin tapis ? Oui, avec le crayon ! À tout à l'heure, Sarah. À tout à l'heure, papa. En ce moment, Sarah s'assoit. Le coin tapis est tiède. Un rayon fait un carré d'or. Les cubes attendent dans leur bac. La maîtresse parle près des chaises. Bonjour les enfants. Bonjour, maîtresse. Sarah veut le crayon, tout de suite. Elle ouvre la boîte trop vite. Le crayon roule sous un cube. Oh. Le sourire de Sarah disparaît. Elle reste près du groupe. Elle reprend le crayon, sans presser. Le bois est râpeux, un peu chaud. Je dessine la maison. Le vert sent le bois. La maison tient sur la feuille. Plus tard, une voix parle trop près. Sarah sent un malaise. Son ventre se serre, tout petit. Elle serre le crayon, puis le pose. Je le dirai à la maison. Le soir, le vestiaire est vide. Le manteau rouge revient. Papa coupe du pain. Ça sent le four. Te voilà. Tu as faim, Sarah ? Sarah veut le dire, tout de suite. Papa, à l'école ! Papa parle à maman, près du pain. Les mots de Sarah se cognent aux leurs. Personne ne tourne la tête. Tu disais quelque chose, Sarah ? Mon ventre s'est serré. Le sourire part, d'un coup. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne sort pas, maman. Ses épaules tombent un peu. Papa s'accroupit à sa hauteur. Tu veux du pain ? Sarah ouvre la bouche.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Sylvain est à l'école. C'est le coin tapis. La maîtresse parle. Sylvain aime &lt;emphasis&gt;écouter&lt;/emphasis&gt;. Il écoute bien. La maîtresse dit : on range. Sylvain range un crayon. Plus tard, un camarade chuchote. Il dit : c'est un secret. Ne le dis pas à la maison. Sylvain sent un malaise. Son ventre est serré. Le soir, papa coupe du pain. Sylvain vient raconter à la maison. Il dit : papa, j'ai un malaise. Maman l'écoute aussi. Papa dit : tu as bien fait. On aime écouter la maîtresse. Si tu as un malaise, tu viens raconter.&lt;/slow&gt; [pause]</t>
+          <t>Le vestiaire sent le pain du goûter. Les crochets portent des prénoms. Le prénom de Sarah est écrit. Un manteau rouge attend dans les bras. Les manches sont un peu froides. Maman lève le manteau vers le crochet. Le métal des crochets luit. Sur le métal, un &lt;emphasis&gt;éclat de crochet&lt;/emphasis&gt; tremble. Il est petit, papa. C'est la lumière, sur le crochet. Papa accroche le manteau rouge. Le crochet tient le tissu. L'éclat de crochet brille, sous le manteau. Tes lacets sont faits, Sarah ? Oui, maman. Maman noue un lacet, puis l'autre. Les chaussures font un petit clac. Tu as senti le pain ? Oui, papa. Il sent le goûter. Sarah tient un crayon vert. Le bois est un peu râpeux. Je veux dessiner, maintenant ! Une maison, au coin tapis ? Oui, avec le crayon ! À tout à l'heure, Sarah. À tout à l'heure, papa. En ce moment, Sarah s'assoit. Le coin tapis est tiède. Un rayon fait un carré d'or. Les cubes attendent dans leur bac. La maîtresse parle près des chaises. Bonjour les enfants. Bonjour, maîtresse. Sarah veut le crayon, tout de suite. Elle ouvre la boîte trop vite. Le crayon roule sous un cube. Oh. Le sourire de Sarah disparaît. Elle reste près du groupe. Elle reprend le crayon, sans presser. Le bois est râpeux, un peu chaud. Je dessine la maison. Le vert sent le bois. La maison tient sur la feuille. Plus tard, une voix parle trop près. Sarah sent un malaise. Son ventre se serre, tout petit. Elle serre le crayon, puis le pose. Je le dirai à la maison. Le soir, le vestiaire est vide. Le manteau rouge revient. Papa coupe du pain. Ça sent le four. Te voilà. Tu as faim, Sarah ? Sarah veut le dire, tout de suite. Papa, à l'école ! Papa parle à maman, près du pain. Les mots de Sarah se cognent aux leurs. Personne ne tourne la tête. Tu disais quelque chose, Sarah ? Mon ventre s'est serré. Le sourire part, d'un coup. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne sort pas, maman. Ses épaules tombent un peu. Papa s'accroupit à sa hauteur. Tu veux du pain ? Sarah ouvre la bouche. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,18 +1246,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>écouter</t>
+          <t>éclat de crochet</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,60 +1324,90 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_dessiner_le_malaise_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un oiseau de papier pose sur la salière.
-narrateur|Le papier fait un petit frou.
-narrateur|Ça sent le pain grillé.
-narrateur|Des miettes dorées sont sur la nappe.
-narrateur|Un rayon touche l'aile pliée.
-narrateur|La salière est un peu froide.
-narrateur|Maman a plié l'oiseau ce matin.
-maman|Il est léger, tu vois ?
+          <t>narrateur|Le vestiaire sent le pain du goûter.
+narrateur|Les crochets portent des prénoms.
+narrateur|Le prénom de Sarah est écrit.
+narrateur|Un manteau rouge attend dans les bras.
+narrateur|Les manches sont un peu froides.
+narrateur|Maman lève le manteau vers le crochet.
+narrateur|Le métal des crochets luit.
+narrateur|Sur le métal, un éclat de crochet tremble.
+enfant-f|Il est petit, papa.
+papa|C'est la lumière, sur le crochet.
+narrateur|Papa accroche le manteau rouge.
+narrateur|Le crochet tient le tissu.
+narrateur|L'éclat de crochet brille, sous le manteau.
+maman|Tes lacets sont faits, Sarah ?
 enfant-f|Oui, maman.
-enfant-f|Je veux lui dessiner une aile.
-enfant-f|Une aile verte.
-papa|Tu pourras à l'école.
-papa|Tu écoutes la maîtresse.
+narrateur|Maman noue un lacet, puis l'autre.
+narrateur|Les chaussures font un petit clac.
+papa|Tu as senti le pain ?
 enfant-f|Oui, papa.
-maman|Les lacets sont bien faits.
+enfant-f|Il sent le goûter.
+narrateur|Sarah tient un crayon vert.
+narrateur|Le bois est un peu râpeux.
+enfant-f|Je veux dessiner, maintenant !
+maman|Une maison, au coin tapis ?
+enfant-f|Oui, avec le crayon !
+papa|À tout à l'heure, Sarah.
+enfant-f|À tout à l'heure, papa.
 narrateur|En ce moment, Sarah s'assoit.
-narrateur|Le tapis a un carré d'or.
-narrateur|Les cubes sont dans leur bac.
-maitresse|On écoute.
-maitresse|Ensuite, on range les crayons.
-narrateur|Sarah aime écouter.
-narrateur|Elle prend un crayon vert.
-narrateur|Le bois est un peu râpeux.
-narrateur|Elle dessine une aile, tout doux.
-narrateur|L'aile a une petite plume.
-narrateur|Le vert sent un peu le bois.
-enfant-f|C'est pour l'oiseau, maîtresse.
-maitresse|Oui, Sarah.
-maitresse|Tu as bien écouté.
-maitresse|On range, maintenant.
-narrateur|Sarah pose le crayon dans la boîte.
-narrateur|L'aile verte reste sur la feuille.
-narrateur|Plus tard, quelqu'un parle tout bas.
-narrateur|Sarah entend parler d'un secret.
-narrateur|Son ventre se serre.
-narrateur|Elle pose la feuille près d'elle.
-enfant-f|Je raconterai à la maison.
-narrateur|Le soir, papa coupe du pain.
-narrateur|La croûte fait un petit bruit.
+narrateur|Le coin tapis est tiède.
+narrateur|Un rayon fait un carré d'or.
+narrateur|Les cubes attendent dans leur bac.
+narrateur|La maîtresse parle près des chaises.
+maitresse|Bonjour les enfants.
+enfant-f|Bonjour, maîtresse.
+narrateur|Sarah veut le crayon, tout de suite.
+narrateur|Elle ouvre la boîte trop vite.
+narrateur|Le crayon roule sous un cube.
+enfant-f|Oh.
+narrateur|Le sourire de Sarah disparaît.
+narrateur|Elle reste près du groupe.
+narrateur|Elle reprend le crayon, sans presser.
+narrateur|Le bois est râpeux, un peu chaud.
+enfant-f|Je dessine la maison.
+narrateur|Le vert sent le bois.
+narrateur|La maison tient sur la feuille.
+narrateur|Plus tard, une voix parle trop près.
+narrateur|Sarah sent un malaise.
+narrateur|Son ventre se serre, tout petit.
+narrateur|Elle serre le crayon, puis le pose.
+enfant-f|Je le dirai à la maison.
+narrateur|Le soir, le vestiaire est vide.
+narrateur|Le manteau rouge revient.
+narrateur|Papa coupe du pain.
 narrateur|Ça sent le four.
+papa|Te voilà.
 papa|Tu as faim, Sarah ?
-narrateur|Sarah vient près de la planche.
-narrateur|Elle a encore le ventre serré.
-narrateur|L'oiseau de papier attend sur la salière.</t>
+narrateur|Sarah veut le dire, tout de suite.
+enfant-f|Papa, à l'école !
+narrateur|Papa parle à maman, près du pain.
+narrateur|Les mots de Sarah se cognent aux leurs.
+narrateur|Personne ne tourne la tête.
+papa|Tu disais quelque chose, Sarah ?
+enfant-f|Mon ventre s'est serré.
+narrateur|Le sourire part, d'un coup.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-f|Ça ne sort pas, maman.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à sa hauteur.
+papa|Tu veux du pain ?
+narrateur|Sarah ouvre la bouche.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>papier,pain</t>
+          <t>vestiaire,manteau</t>
         </is>
       </c>
     </row>
@@ -1409,22 +1439,22 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sylvain a un malaise. Que fait-il ?&lt;/prosody&gt;&lt;break time="250ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah a un &lt;emphasis level="moderate"&gt;malaise&lt;/emphasis&gt;. Que fait-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Sylvain a un malaise. Que fait-il ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Sarah a un &lt;emphasis&gt;malaise&lt;/emphasis&gt;. Que fait-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>raconter</t>
+          <t>elle raconte</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>raconter | elle raconte | à papa | à la maison | écouter</t>
+          <t>elle raconte | raconter | au goûter | au gouter | à papa | à la maison | elle attend | elle dit | papa | malaise</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1439,7 +1469,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Elle raconte à papa. Que fait Sarah ?</t>
+          <t>Sarah a un malaise. Elle raconte au goûter. Que fait-elle ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1477,7 +1507,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1485,10 +1515,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1503,34 +1533,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>malaise</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1539,13 +1573,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1555,7 +1589,7 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_raconte_au_gouter; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1588,17 +1622,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Papa, j'ai un malaise. Quelqu'un a parlé d'un secret. Maman pose le beurre. Tu as bien fait de raconter. On aime écouter la maîtresse. Si tu as un malaise, tu viens raconter. À papa ou à maman. Sarah respire. J'ai dessiné une aile verte. On la colle sur l'oiseau ? Oui. Papa prend la feuille. L'aile est un peu recourbée. Il la pose près du papier plié. Elle va bien, là ? Un peu plus près du bec.</t>
+          <t>Sarah ouvre la bouche trop vite. Papa, à l'école, quelqu'un parlait ! Papa n'a pas fini sa phrase. Le pain, sur la planche, Sarah. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme la bouche. Elle pose les mains à plat. Elle écoute la maison, un instant. Le goûter est près de la fenêtre. Papa pose un verre d'eau. Maman pose le pain. Sarah attend que le silence arrive. Sur le crochet, l'éclat de crochet brille. Je peux te dire quelque chose ? Oui, nous t'écoutons. À l'école, quelqu'un a parlé trop près. Mon ventre s'est serré. Merci, Sarah. Papa a entendu toute la phrase. Tu as soif ? Un peu, maman. Le ventre de Sarah se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sylvain a écouté la maîtresse. Il a raconté son malaise à la maison. Papa et maman sont là.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah ouvre la bouche trop vite. Papa, à l'école, quelqu'un parlait ! Papa n'a pas fini sa phrase. Le pain, sur la planche, Sarah. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme la bouche. Elle pose les mains à plat. Elle écoute la maison, un instant. Le &lt;emphasis level="moderate"&gt;goûter&lt;/emphasis&gt; est près de la fenêtre. Papa pose un verre d'eau. Maman pose le pain. Sarah attend que le silence arrive. Sur le crochet, l'éclat de crochet brille. Je peux te dire quelque chose ? Oui, nous t'écoutons. À l'école, quelqu'un a parlé trop près. Mon ventre s'est serré. Merci, Sarah. Papa a entendu toute la phrase. Tu as soif ? Un peu, maman. Le ventre de Sarah se desserre.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Sylvain a écouté la maîtresse. Il a raconté son malaise à la maison. Papa et maman sont là.&lt;/slow&gt; [pause]</t>
+          <t>Sarah ouvre la bouche trop vite. Papa, à l'école, quelqu'un parlait ! Papa n'a pas fini sa phrase. Le pain, sur la planche, Sarah. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme la bouche. Elle pose les mains à plat. Elle écoute la maison, un instant. Le &lt;emphasis&gt;goûter&lt;/emphasis&gt; est près de la fenêtre. Papa pose un verre d'eau. Maman pose le pain. Sarah attend que le silence arrive. Sur le crochet, l'éclat de crochet brille. Je peux te dire quelque chose ? Oui, nous t'écoutons. À l'école, quelqu'un a parlé trop près. Mon ventre s'est serré. Merci, Sarah. Papa a entendu toute la phrase. Tu as soif ? Un peu, maman. Le ventre de Sarah se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1645,18 +1679,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1677,28 +1711,32 @@
       <c r="AG4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr">
+        <is>
+          <t>goûter</t>
+        </is>
+      </c>
       <c r="AI4" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ4" s="2" t="n">
         <v>450</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>280</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1707,10 +1745,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1719,31 +1757,45 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=soulagement_prudent; intensite=1; destinataire=enfant; sous_texte=elle_refuse_de_foncer_puis_raconte; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>enfant-f|Papa, j'ai un malaise.
-enfant-f|Quelqu'un a parlé d'un secret.
-narrateur|Maman pose le beurre.
-maman|Tu as bien fait de raconter.
-maman|On aime écouter la maîtresse.
-papa|Si tu as un malaise, tu viens raconter.
-papa|À papa ou à maman.
-narrateur|Sarah respire.
-enfant-f|J'ai dessiné une aile verte.
-maman|On la colle sur l'oiseau ?
-enfant-f|Oui.
-narrateur|Papa prend la feuille.
-narrateur|L'aile est un peu recourbée.
-narrateur|Il la pose près du papier plié.
-papa|Elle va bien, là ?
-enfant-f|Un peu plus près du bec.</t>
+          <t>narrateur|Sarah ouvre la bouche trop vite.
+enfant-f|Papa, à l'école, quelqu'un parlait !
+narrateur|Papa n'a pas fini sa phrase.
+papa|Le pain, sur la planche, Sarah.
+narrateur|Les deux voix se mélangent.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Sarah refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Elle pose les mains à plat.
+narrateur|Elle écoute la maison, un instant.
+maman|Le goûter est près de la fenêtre.
+narrateur|Papa pose un verre d'eau.
+narrateur|Maman pose le pain.
+narrateur|Sarah attend que le silence arrive.
+narrateur|Sur le crochet, l'éclat de crochet brille.
+enfant-f|Je peux te dire quelque chose ?
+maman|Oui, nous t'écoutons.
+enfant-f|À l'école, quelqu'un a parlé trop près.
+enfant-f|Mon ventre s'est serré.
+papa|Merci, Sarah.
+narrateur|Papa a entendu toute la phrase.
+maman|Tu as soif ?
+enfant-f|Un peu, maman.
+narrateur|Le ventre de Sarah se desserre.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>pain,verre</t>
         </is>
       </c>
     </row>
@@ -1770,17 +1822,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Maman tient l'oiseau. L'aile verte le rejoint. Il peut partir. Je te tiens la main ? Oui, papa. Sa main est chaude. Tu veux un bout de pain ? Oui, maman. La mie est toute douce. Papa verse un verre d'eau. Sarah boit une gorgée. L'oiseau reste près de la salière.</t>
+          <t>Sarah range son crayon près de la porte. On s'assoit près de la fenêtre ? Oui. On voit le manteau rouge. Le pain est tiède, un peu doré. Il sent le goûter, maman. Tes pieds sont sous la table ? Oui, maman. Sarah veut raconter l'école, d'un coup. Elle saisit le crayon trop vite. Le crayon roule vers le pain. Oh. Les mots se bousculent dans sa bouche. Attends. Elle refuse de foncer. Elle reprend le crayon, sans presser. Le coin tapis était tiède. J'ai dessiné la maison. Avec le crayon vert ? Oui, et l'éclat était là. Sarah croque le pain. Une miette reste sur le doigt. Il est bon ? Oui, maman.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sylvain boit un verre d'eau. Papa lui tient la &lt;emphasis level="moderate"&gt;main&lt;/emphasis&gt;.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah range son crayon près de la porte. On s'assoit près de la fenêtre ? Oui. On voit le manteau rouge. Le pain est tiède, un peu doré. Il sent le goûter, maman. Tes pieds sont sous la table ? Oui, maman. Sarah veut raconter l'école, d'un coup. Elle saisit le crayon trop vite. Le crayon roule vers le pain. Oh. Les mots se bousculent dans sa bouche. Attends. Elle refuse de foncer. Elle reprend le crayon, sans presser. Le coin tapis était tiède. J'ai dessiné la maison. Avec le crayon vert ? Oui, et l'éclat était là. Sarah croque le pain. Une miette reste sur le doigt. Il est bon ? Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Sylvain boit un verre d'eau. Papa lui tient la &lt;emphasis&gt;main&lt;/emphasis&gt;.&lt;/slow&gt; [pause]</t>
+          <t>Sarah range son crayon près de la porte. On s'assoit près de la fenêtre ? Oui. On voit le manteau rouge. Le pain est tiède, un peu doré. Il sent le goûter, maman. Tes pieds sont sous la table ? Oui, maman. Sarah veut raconter l'école, d'un coup. Elle saisit le crayon trop vite. Le crayon roule vers le pain. Oh. Les mots se bousculent dans sa bouche. Attends. Elle refuse de foncer. Elle reprend le crayon, sans presser. Le coin tapis était tiède. J'ai dessiné la maison. Avec le crayon vert ? Oui, et l'éclat était là. Sarah croque le pain. Une miette reste sur le doigt. Il est bon ? Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1827,18 +1879,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.14</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1865,26 +1917,26 @@
         </is>
       </c>
       <c r="AI5" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1893,10 +1945,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1905,28 +1957,44 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=résolution; intention=faire_vivre_la_réussite; emotion=fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_l_eclat_tient; tempo=naturel; sourire=franc; respiration=relâchée</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Maman tient l'oiseau.
-narrateur|L'aile verte le rejoint.
-enfant-f|Il peut partir.
-papa|Je te tiens la main ?
-enfant-f|Oui, papa.
-narrateur|Sa main est chaude.
-maman|Tu veux un bout de pain ?
+          <t>narrateur|Sarah range son crayon près de la porte.
+papa|On s'assoit près de la fenêtre ?
+enfant-f|Oui.
+narrateur|On voit le manteau rouge.
+narrateur|Le pain est tiède, un peu doré.
+enfant-f|Il sent le goûter, maman.
+maman|Tes pieds sont sous la table ?
 enfant-f|Oui, maman.
-narrateur|La mie est toute douce.
-narrateur|Papa verse un verre d'eau.
-narrateur|Sarah boit une gorgée.
-narrateur|L'oiseau reste près de la salière.</t>
+narrateur|Sarah veut raconter l'école, d'un coup.
+narrateur|Elle saisit le crayon trop vite.
+narrateur|Le crayon roule vers le pain.
+enfant-f|Oh.
+narrateur|Les mots se bousculent dans sa bouche.
+enfant-f|Attends.
+narrateur|Elle refuse de foncer.
+narrateur|Elle reprend le crayon, sans presser.
+enfant-f|Le coin tapis était tiède.
+enfant-f|J'ai dessiné la maison.
+papa|Avec le crayon vert ?
+enfant-f|Oui, et l'éclat était là.
+narrateur|Sarah croque le pain.
+narrateur|Une miette reste sur le doigt.
+maman|Il est bon ?
+enfant-f|Oui, maman.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>verre,pain</t>
+          <t>pain,crayon</t>
         </is>
       </c>
     </row>
@@ -1953,17 +2021,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>L'oiseau a son aile. J'ai écouté. J'ai raconté. On t'a écoutée. Bravo, Sarah.</t>
+          <t>Le manteau rouge est rentré. Il pend, près de la porte. Le crochet de la maison garde un peu de lumière. Comme à l'école, papa ! Tu le vois, toi ? Oui, sur le métal. Le pain du goûter attend sur la planche. On est bien, ici. Le crayon est rangé ? Près de la porte, maman. Sarah pose la miette dans la coupelle. L'éclat de crochet tient sur le métal.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>L'oiseau a son aile. J'ai écouté. J'ai raconté. On t'a écoutée. Bravo, Sarah.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le manteau rouge est rentré. Il pend, près de la porte. Le crochet de la maison garde un peu de lumière. Comme à l'école, papa ! Tu le vois, toi ? Oui, sur le métal. Le pain du goûter attend sur la planche. On est bien, ici. Le crayon est rangé ? Près de la porte, maman. Sarah pose la miette dans la coupelle. L'&lt;emphasis level="moderate"&gt;éclat de crochet&lt;/emphasis&gt; tient sur le métal.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le manteau rouge est rentré. Il pend, près de la porte. Le crochet de la maison garde un peu de lumière. Comme à l'école, papa ! Tu le vois, toi ? Oui, sur le métal. Le pain du goûter attend sur la planche. On est bien, ici. Le crayon est rangé ? Près de la porte, maman. Sarah pose la miette dans la coupelle. L'&lt;emphasis&gt;éclat de crochet&lt;/emphasis&gt; tient sur le métal.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2010,7 +2078,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2018,10 +2086,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.36</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2030,12 +2098,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2044,17 +2112,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de crochet</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2063,11 +2135,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2076,28 +2148,44 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_tient_sur_le_metal; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|L'oiseau a son aile.
-enfant-f|J'ai écouté.
-enfant-f|J'ai raconté.
-maman|On t'a écoutée.
-papa|Bravo, Sarah.</t>
+          <t>enfant-f|Le manteau rouge est rentré.
+maman|Il pend, près de la porte.
+narrateur|Le crochet de la maison garde un peu de lumière.
+enfant-f|Comme à l'école, papa !
+papa|Tu le vois, toi ?
+enfant-f|Oui, sur le métal.
+narrateur|Le pain du goûter attend sur la planche.
+enfant-f|On est bien, ici.
+maman|Le crayon est rangé ?
+enfant-f|Près de la porte, maman.
+narrateur|Sarah pose la miette dans la coupelle.
+narrateur|L'éclat de crochet tient sur le métal.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>manteau,crochet</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2203,6 +2291,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>